<commit_message>
minor updates for releve
</commit_message>
<xml_diff>
--- a/Data_Workflow_3_Final_Polishing/Data_dictionaries/releve_dictionary_ms.xlsx
+++ b/Data_Workflow_3_Final_Polishing/Data_dictionaries/releve_dictionary_ms.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henryfrye/Dropbox/Intellectual_Endeavours/DimensionsDataPaper/GCFR_Traits/Data_Workflow_3_Final_Polishing/Data_dictionaries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41781240-C48B-5442-BC56-074DF90962B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BDA1B1-8077-664F-B769-93844BED3C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="16020" xr2:uid="{9F7D886F-24CC-3247-8AC7-DE51D29761AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
   <si>
     <t>Column.Name</t>
   </si>
@@ -165,6 +165,27 @@
   </si>
   <si>
     <t>The percent cover relative to the total plot percent cover</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>longitude</t>
+  </si>
+  <si>
+    <t>18.374421 - 24.4833</t>
+  </si>
+  <si>
+    <t>Latitude of plot location</t>
+  </si>
+  <si>
+    <t>Longitude of plot location</t>
+  </si>
+  <si>
+    <t>Decimal degrees</t>
+  </si>
+  <si>
+    <t>-34.4 - -30.3925</t>
   </si>
 </sst>
 </file>
@@ -200,11 +221,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -539,11 +561,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD17FC8-F08D-DD47-A2FC-504B7EE9547E}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="4" max="4" width="32.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -706,58 +729,58 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" t="s">
-        <v>24</v>
+      <c r="D9" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="F9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="221" x14ac:dyDescent="0.2">
+        <v>1566</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="F10">
-        <v>10670</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
         <v>38</v>
@@ -766,23 +789,63 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="221" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12">
+        <v>10670</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C14" t="s">
         <v>23</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D14" t="s">
         <v>30</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E14" t="s">
         <v>38</v>
       </c>
-      <c r="F12">
+      <c r="F14">
         <v>0</v>
       </c>
     </row>

</xml_diff>